<commit_message>
MACD scan results 2026-09-29
</commit_message>
<xml_diff>
--- a/results/macd_2026-09-29.xlsx
+++ b/results/macd_2026-09-29.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>NTES</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,19 +462,19 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ALAB</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NTES</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>ACLS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -485,30 +485,26 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
+          <t>AMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AEIS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>AEHR</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>REG</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ACLS</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>AMRX</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>APPS</t>
         </is>
       </c>
     </row>
@@ -521,13 +517,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>ARCC</t>
         </is>
       </c>
     </row>
@@ -535,18 +531,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ARW</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
@@ -554,18 +550,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BATRK</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>ARW</t>
         </is>
       </c>
     </row>
@@ -573,18 +569,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AXTI</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
@@ -592,18 +588,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>FELE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BLFS</t>
+          <t>DIOD</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BAND</t>
+          <t>AVT</t>
         </is>
       </c>
     </row>
@@ -611,18 +607,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>BAND</t>
         </is>
       </c>
     </row>
@@ -630,18 +626,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>BLFS</t>
         </is>
       </c>
     </row>
@@ -649,18 +645,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LUNR</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BRKR</t>
         </is>
       </c>
     </row>
@@ -668,18 +664,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>NVMI</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DGII</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
@@ -687,18 +683,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>NVTS</t>
+          <t>NVMI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>IOVA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DIOD</t>
+          <t>CHEF</t>
         </is>
       </c>
     </row>
@@ -706,18 +702,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>NVTS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>DXPE</t>
+          <t>COHU</t>
         </is>
       </c>
     </row>
@@ -725,7 +721,7 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -736,7 +732,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>EMBJ</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -744,7 +740,7 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -755,7 +751,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
@@ -763,18 +759,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>POET</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>LAUR</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ETON</t>
+          <t>EMBJ</t>
         </is>
       </c>
     </row>
@@ -782,18 +778,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SHMD</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
@@ -801,48 +797,56 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>RYAAY</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LTRX</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>LFUS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>STRL</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>MGNI</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>MRNA</t>
         </is>
       </c>
     </row>
@@ -851,13 +855,13 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NNBR</t>
+          <t>LTRX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>IRDM</t>
+          <t>MRVL</t>
         </is>
       </c>
     </row>
@@ -866,13 +870,13 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>MSFT</t>
         </is>
       </c>
     </row>
@@ -881,13 +885,13 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>MU</t>
         </is>
       </c>
     </row>
@@ -896,13 +900,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>MTSI</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
@@ -911,13 +915,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>MXL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>MTSI</t>
+          <t>OUST</t>
         </is>
       </c>
     </row>
@@ -926,13 +930,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>NDSN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>MXL</t>
+          <t>PLXS</t>
         </is>
       </c>
     </row>
@@ -941,13 +945,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>NNBR</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>PRTH</t>
         </is>
       </c>
     </row>
@@ -956,13 +960,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>RGEN</t>
         </is>
       </c>
     </row>
@@ -971,13 +975,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>QMCO</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PGEN</t>
+          <t>ROST</t>
         </is>
       </c>
     </row>
@@ -986,13 +990,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>RXT</t>
         </is>
       </c>
     </row>
@@ -1001,13 +1005,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SATL</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PLXS</t>
+          <t>SANM</t>
         </is>
       </c>
     </row>
@@ -1016,13 +1020,13 @@
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SITM</t>
+          <t>PGEN</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>SATL</t>
         </is>
       </c>
     </row>
@@ -1031,13 +1035,13 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SONO</t>
+          <t>QMCO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>SIMO</t>
         </is>
       </c>
     </row>
@@ -1046,13 +1050,13 @@
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>SHOO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>SKYW</t>
         </is>
       </c>
     </row>
@@ -1061,13 +1065,13 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
@@ -1076,31 +1080,39 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>SITM</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>SIMO</t>
+          <t>SMTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SRZN</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>SONO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
@@ -1111,11 +1123,15 @@
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>TEM</t>
         </is>
       </c>
     </row>
@@ -1141,17 +1157,6 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>